<commit_message>
Add pen mins to box stats
</commit_message>
<xml_diff>
--- a/Test_Data/FactTable.xlsx
+++ b/Test_Data/FactTable.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/55cd0139eebd0c53/Desktop/Github Repo/PaupackLaxStatTracking/Test_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B0F9D27-3A12-462D-A569-EF3945346ED1}"/>
+  <xr:revisionPtr revIDLastSave="341" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71565E1A-B9F7-4D40-82F5-248252D4BA31}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5010" windowWidth="29040" windowHeight="15720" xr2:uid="{FADB34D3-2AD0-4900-91AC-1DDA22919594}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   </externalReferences>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId4"/>
+    <pivotCache cacheId="6" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="60">
   <si>
     <t>Maplewood HS</t>
   </si>
@@ -194,15 +194,42 @@
   <si>
     <t>Sum of Assists</t>
   </si>
+  <si>
+    <t>Sum of GBs</t>
+  </si>
+  <si>
+    <t>Sum of CTOs</t>
+  </si>
+  <si>
+    <t>Sum of TOs</t>
+  </si>
+  <si>
+    <t>Sum of WomanUpGoals</t>
+  </si>
+  <si>
+    <t>Sum of WomanDownGoals</t>
+  </si>
+  <si>
+    <t>Sum of Shots</t>
+  </si>
+  <si>
+    <t>Sum of ShotsFaced</t>
+  </si>
+  <si>
+    <t>Sum of Saves</t>
+  </si>
+  <si>
+    <t>Sum of DrawAtts</t>
+  </si>
+  <si>
+    <t>Sum of DrawControls</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="170" formatCode="0.0%"/>
-  </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -220,23 +247,8 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -255,14 +267,8 @@
         <bgColor rgb="FF1F4E79"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -285,21 +291,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -315,12 +311,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -494,7 +487,14 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="11"/>
     </cacheField>
     <cacheField name="Saves" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="8"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="8" count="6">
+        <n v="0"/>
+        <n v="4"/>
+        <n v="3"/>
+        <n v="8"/>
+        <n v="1"/>
+        <n v="5"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="WomanUpGoals" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
@@ -506,7 +506,13 @@
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
     </cacheField>
     <cacheField name="PenType" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+      <sharedItems containsBlank="1" count="5">
+        <m/>
+        <s v="Green"/>
+        <s v="Yellow"/>
+        <s v="12m"/>
+        <s v="Red"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="MinsServed" numFmtId="0">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
@@ -535,11 +541,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -555,11 +561,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -575,11 +581,11 @@
     <n v="4"/>
     <n v="3"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -595,11 +601,11 @@
     <n v="3"/>
     <n v="2"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -615,11 +621,11 @@
     <n v="2"/>
     <n v="2"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -635,11 +641,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -655,11 +661,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="0"/>
     <n v="3"/>
-    <s v="Green"/>
+    <x v="1"/>
     <n v="1"/>
   </r>
   <r>
@@ -675,11 +681,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -695,11 +701,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -715,11 +721,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="5"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -735,11 +741,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -755,11 +761,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -775,11 +781,11 @@
     <n v="4"/>
     <n v="3"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -795,11 +801,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -815,11 +821,11 @@
     <n v="4"/>
     <n v="2"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -835,11 +841,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -855,11 +861,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -875,11 +881,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <s v="Green"/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="1"/>
     <n v="1"/>
   </r>
   <r>
@@ -895,11 +901,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="0"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -915,11 +921,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="8"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="1"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -935,11 +941,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <s v="Yellow"/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="2"/>
     <n v="1"/>
   </r>
   <r>
@@ -955,11 +961,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -975,11 +981,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -995,11 +1001,11 @@
     <n v="1"/>
     <n v="1"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1015,11 +1021,11 @@
     <n v="3"/>
     <n v="3"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1035,11 +1041,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1055,11 +1061,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1075,11 +1081,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1095,11 +1101,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1115,11 +1121,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="9"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <s v="Green"/>
+    <x v="2"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="1"/>
     <n v="1"/>
   </r>
   <r>
@@ -1135,11 +1141,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <s v="12m"/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="3"/>
     <n v="0"/>
   </r>
   <r>
@@ -1155,11 +1161,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <s v="Yellow"/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="2"/>
     <n v="1"/>
   </r>
   <r>
@@ -1175,11 +1181,11 @@
     <n v="4"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1195,11 +1201,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1215,11 +1221,11 @@
     <n v="3"/>
     <n v="1"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1235,11 +1241,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1255,11 +1261,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1275,11 +1281,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1295,11 +1301,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1315,11 +1321,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="8"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="2"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1335,11 +1341,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1355,11 +1361,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1375,11 +1381,11 @@
     <n v="1"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1395,11 +1401,11 @@
     <n v="4"/>
     <n v="3"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1415,11 +1421,11 @@
     <n v="1"/>
     <n v="1"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1435,11 +1441,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="0"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1455,11 +1461,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <s v="Green"/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="1"/>
     <n v="0"/>
   </r>
   <r>
@@ -1475,11 +1481,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="1"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1495,11 +1501,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1515,11 +1521,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="11"/>
-    <n v="8"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="3"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1535,11 +1541,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1555,11 +1561,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <s v="12m"/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="3"/>
     <n v="0"/>
   </r>
   <r>
@@ -1575,11 +1581,11 @@
     <n v="2"/>
     <n v="2"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1595,11 +1601,11 @@
     <n v="4"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1615,11 +1621,11 @@
     <n v="3"/>
     <n v="1"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1635,11 +1641,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1655,11 +1661,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="0"/>
     <n v="3"/>
-    <s v="Yellow"/>
+    <x v="2"/>
     <n v="1"/>
   </r>
   <r>
@@ -1675,11 +1681,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="1"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1695,11 +1701,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1715,11 +1721,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="5"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <s v="12m"/>
+    <x v="4"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="3"/>
     <n v="0"/>
   </r>
   <r>
@@ -1735,11 +1741,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <s v="Yellow"/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="2"/>
     <n v="1"/>
   </r>
   <r>
@@ -1755,11 +1761,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1775,11 +1781,11 @@
     <n v="2"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1795,11 +1801,11 @@
     <n v="1"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <s v="Red"/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="4"/>
     <n v="0"/>
   </r>
   <r>
@@ -1815,11 +1821,11 @@
     <n v="1"/>
     <n v="1"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="2"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1835,11 +1841,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="1"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1855,11 +1861,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="0"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1875,11 +1881,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <m/>
+    <x v="0"/>
+    <n v="0"/>
+    <n v="1"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1895,11 +1901,11 @@
     <n v="0"/>
     <n v="0"/>
     <n v="0"/>
-    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
     <n v="1"/>
     <n v="3"/>
-    <m/>
+    <x v="0"/>
     <n v="0"/>
   </r>
   <r>
@@ -1915,19 +1921,19 @@
     <n v="0"/>
     <n v="0"/>
     <n v="10"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <m/>
+    <x v="5"/>
+    <n v="0"/>
+    <n v="0"/>
+    <n v="0"/>
+    <x v="0"/>
     <n v="0"/>
   </r>
 </pivotCacheRecords>
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{93B1F2E5-6101-4B7D-8463-217B5EDC7EF7}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:C14" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{93B1F2E5-6101-4B7D-8463-217B5EDC7EF7}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A3:M14" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="18">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -1960,17 +1966,36 @@
     <pivotField showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
     <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0">
+      <items count="7">
+        <item x="0"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="3"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
   </pivotFields>
   <rowFields count="1">
@@ -2014,17 +2039,57 @@
   <colFields count="1">
     <field x="-2"/>
   </colFields>
-  <colItems count="2">
+  <colItems count="12">
     <i>
       <x/>
     </i>
     <i i="1">
       <x v="1"/>
     </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+    <i i="5">
+      <x v="5"/>
+    </i>
+    <i i="6">
+      <x v="6"/>
+    </i>
+    <i i="7">
+      <x v="7"/>
+    </i>
+    <i i="8">
+      <x v="8"/>
+    </i>
+    <i i="9">
+      <x v="9"/>
+    </i>
+    <i i="10">
+      <x v="10"/>
+    </i>
+    <i i="11">
+      <x v="11"/>
+    </i>
   </colItems>
-  <dataFields count="2">
+  <dataFields count="12">
     <dataField name="Sum of Goals" fld="4" baseField="0" baseItem="0"/>
     <dataField name="Sum of Assists" fld="5" baseField="0" baseItem="0"/>
+    <dataField name="Sum of GBs" fld="7" baseField="0" baseItem="0"/>
+    <dataField name="Sum of TOs" fld="8" baseField="0" baseItem="0"/>
+    <dataField name="Sum of CTOs" fld="15" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Shots" fld="6" baseField="0" baseItem="0"/>
+    <dataField name="Sum of WomanUpGoals" fld="13" baseField="0" baseItem="0"/>
+    <dataField name="Sum of WomanDownGoals" fld="14" baseField="0" baseItem="0"/>
+    <dataField name="Sum of DrawAtts" fld="9" baseField="0" baseItem="0"/>
+    <dataField name="Sum of DrawControls" fld="10" baseField="0" baseItem="0"/>
+    <dataField name="Sum of ShotsFaced" fld="11" baseField="0" baseItem="0"/>
+    <dataField name="Sum of Saves" fld="12" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -2355,29 +2420,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EBA3C68-2291-42D7-93ED-B36167695E1B}">
-  <dimension ref="A3:F14"/>
+  <dimension ref="A3:M14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.26953125" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6328125" hidden="1" customWidth="1"/>
-    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="24.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>46</v>
       </c>
@@ -2387,14 +2448,38 @@
       <c r="C3" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G3" t="s">
+        <v>55</v>
+      </c>
+      <c r="H3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J3" t="s">
+        <v>58</v>
+      </c>
+      <c r="K3" t="s">
+        <v>59</v>
+      </c>
+      <c r="L3" t="s">
+        <v>56</v>
+      </c>
+      <c r="M3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>40</v>
       </c>
@@ -2405,17 +2490,37 @@
         <v>4</v>
       </c>
       <c r="D4" s="6">
+        <v>20</v>
+      </c>
+      <c r="E4" s="6">
         <v>6</v>
       </c>
-      <c r="E4" s="6">
-        <v>4</v>
-      </c>
-      <c r="F4" s="8">
-        <f>+D4/SUM(D4:E4)</f>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="F4" s="6">
+        <v>9</v>
+      </c>
+      <c r="G4" s="6">
+        <v>17</v>
+      </c>
+      <c r="H4" s="6">
+        <v>1</v>
+      </c>
+      <c r="I4" s="6">
+        <v>0</v>
+      </c>
+      <c r="J4" s="6">
+        <v>17</v>
+      </c>
+      <c r="K4" s="6">
+        <v>11</v>
+      </c>
+      <c r="L4" s="6">
+        <v>0</v>
+      </c>
+      <c r="M4" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="5" t="s">
         <v>41</v>
       </c>
@@ -2426,17 +2531,37 @@
         <v>3</v>
       </c>
       <c r="D5" s="6">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="E5" s="6">
+        <v>9</v>
+      </c>
+      <c r="F5" s="6">
+        <v>11</v>
+      </c>
+      <c r="G5" s="6">
+        <v>11</v>
+      </c>
+      <c r="H5" s="6">
+        <v>0</v>
+      </c>
+      <c r="I5" s="6">
         <v>3</v>
       </c>
-      <c r="F5" s="8">
-        <f t="shared" ref="F5:F13" si="0">+D5/SUM(D5:E5)</f>
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="J5" s="6">
+        <v>0</v>
+      </c>
+      <c r="K5" s="6">
+        <v>0</v>
+      </c>
+      <c r="L5" s="6">
+        <v>0</v>
+      </c>
+      <c r="M5" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>38</v>
       </c>
@@ -2447,17 +2572,37 @@
         <v>8</v>
       </c>
       <c r="D6" s="6">
+        <v>18</v>
+      </c>
+      <c r="E6" s="6">
+        <v>5</v>
+      </c>
+      <c r="F6" s="6">
+        <v>4</v>
+      </c>
+      <c r="G6" s="6">
+        <v>16</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0</v>
+      </c>
+      <c r="J6" s="6">
+        <v>17</v>
+      </c>
+      <c r="K6" s="6">
         <v>8</v>
       </c>
-      <c r="E6" s="6">
-        <v>8</v>
-      </c>
-      <c r="F6" s="8">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="L6" s="6">
+        <v>0</v>
+      </c>
+      <c r="M6" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="5" t="s">
         <v>43</v>
       </c>
@@ -2468,17 +2613,37 @@
         <v>3</v>
       </c>
       <c r="D7" s="6">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="E7" s="6">
+        <v>8</v>
+      </c>
+      <c r="F7" s="6">
+        <v>11</v>
+      </c>
+      <c r="G7" s="6">
+        <v>13</v>
+      </c>
+      <c r="H7" s="6">
+        <v>0</v>
+      </c>
+      <c r="I7" s="6">
         <v>3</v>
       </c>
-      <c r="F7" s="8">
-        <f t="shared" si="0"/>
-        <v>0.66666666666666663</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="J7" s="6">
+        <v>0</v>
+      </c>
+      <c r="K7" s="6">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6">
+        <v>0</v>
+      </c>
+      <c r="M7" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="5" t="s">
         <v>45</v>
       </c>
@@ -2489,17 +2654,37 @@
         <v>0</v>
       </c>
       <c r="D8" s="6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E8" s="6">
-        <v>0</v>
-      </c>
-      <c r="F8" s="8" t="e">
-        <f t="shared" si="0"/>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="F8" s="6">
+        <v>0</v>
+      </c>
+      <c r="G8" s="6">
+        <v>0</v>
+      </c>
+      <c r="H8" s="6">
+        <v>0</v>
+      </c>
+      <c r="I8" s="6">
+        <v>0</v>
+      </c>
+      <c r="J8" s="6">
+        <v>0</v>
+      </c>
+      <c r="K8" s="6">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6">
+        <v>56</v>
+      </c>
+      <c r="M8" s="6">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="5" t="s">
         <v>37</v>
       </c>
@@ -2510,17 +2695,37 @@
         <v>8</v>
       </c>
       <c r="D9" s="6">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E9" s="6">
-        <v>8</v>
-      </c>
-      <c r="F9" s="8">
-        <f t="shared" si="0"/>
-        <v>0.46666666666666667</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+        <v>9</v>
+      </c>
+      <c r="F9" s="6">
+        <v>4</v>
+      </c>
+      <c r="G9" s="6">
+        <v>21</v>
+      </c>
+      <c r="H9" s="6">
+        <v>2</v>
+      </c>
+      <c r="I9" s="6">
+        <v>0</v>
+      </c>
+      <c r="J9" s="6">
+        <v>0</v>
+      </c>
+      <c r="K9" s="6">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6">
+        <v>0</v>
+      </c>
+      <c r="M9" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>44</v>
       </c>
@@ -2531,17 +2736,37 @@
         <v>2</v>
       </c>
       <c r="D10" s="6">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E10" s="6">
-        <v>2</v>
-      </c>
-      <c r="F10" s="8">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="F10" s="6">
+        <v>11</v>
+      </c>
+      <c r="G10" s="6">
+        <v>9</v>
+      </c>
+      <c r="H10" s="6">
+        <v>0</v>
+      </c>
+      <c r="I10" s="6">
+        <v>4</v>
+      </c>
+      <c r="J10" s="6">
+        <v>0</v>
+      </c>
+      <c r="K10" s="6">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6">
+        <v>0</v>
+      </c>
+      <c r="M10" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="5" t="s">
         <v>36</v>
       </c>
@@ -2552,17 +2777,37 @@
         <v>5</v>
       </c>
       <c r="D11" s="6">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="E11" s="6">
-        <v>5</v>
-      </c>
-      <c r="F11" s="8">
-        <f t="shared" si="0"/>
-        <v>0.73684210526315785</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="F11" s="6">
+        <v>3</v>
+      </c>
+      <c r="G11" s="6">
+        <v>26</v>
+      </c>
+      <c r="H11" s="6">
+        <v>2</v>
+      </c>
+      <c r="I11" s="6">
+        <v>0</v>
+      </c>
+      <c r="J11" s="6">
+        <v>0</v>
+      </c>
+      <c r="K11" s="6">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6">
+        <v>0</v>
+      </c>
+      <c r="M11" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="5" t="s">
         <v>42</v>
       </c>
@@ -2573,17 +2818,37 @@
         <v>2</v>
       </c>
       <c r="D12" s="6">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E12" s="6">
-        <v>2</v>
-      </c>
-      <c r="F12" s="8">
-        <f t="shared" si="0"/>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+        <v>10</v>
+      </c>
+      <c r="F12" s="6">
+        <v>13</v>
+      </c>
+      <c r="G12" s="6">
+        <v>7</v>
+      </c>
+      <c r="H12" s="6">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6">
+        <v>2</v>
+      </c>
+      <c r="J12" s="6">
+        <v>0</v>
+      </c>
+      <c r="K12" s="6">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6">
+        <v>0</v>
+      </c>
+      <c r="M12" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="5" t="s">
         <v>39</v>
       </c>
@@ -2594,17 +2859,37 @@
         <v>9</v>
       </c>
       <c r="D13" s="6">
+        <v>17</v>
+      </c>
+      <c r="E13" s="6">
+        <v>12</v>
+      </c>
+      <c r="F13" s="6">
         <v>6</v>
       </c>
-      <c r="E13" s="6">
-        <v>9</v>
-      </c>
-      <c r="F13" s="8">
-        <f t="shared" si="0"/>
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="G13" s="6">
+        <v>14</v>
+      </c>
+      <c r="H13" s="6">
+        <v>0</v>
+      </c>
+      <c r="I13" s="6">
+        <v>0</v>
+      </c>
+      <c r="J13" s="6">
+        <v>13</v>
+      </c>
+      <c r="K13" s="6">
+        <v>6</v>
+      </c>
+      <c r="L13" s="6">
+        <v>0</v>
+      </c>
+      <c r="M13" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="5" t="s">
         <v>47</v>
       </c>
@@ -2613,6 +2898,36 @@
       </c>
       <c r="C14" s="6">
         <v>44</v>
+      </c>
+      <c r="D14" s="6">
+        <v>170</v>
+      </c>
+      <c r="E14" s="6">
+        <v>79</v>
+      </c>
+      <c r="F14" s="6">
+        <v>72</v>
+      </c>
+      <c r="G14" s="6">
+        <v>134</v>
+      </c>
+      <c r="H14" s="6">
+        <v>5</v>
+      </c>
+      <c r="I14" s="6">
+        <v>12</v>
+      </c>
+      <c r="J14" s="6">
+        <v>47</v>
+      </c>
+      <c r="K14" s="6">
+        <v>25</v>
+      </c>
+      <c r="L14" s="6">
+        <v>56</v>
+      </c>
+      <c r="M14" s="6">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert changes to test data files
</commit_message>
<xml_diff>
--- a/Test_Data/FactTable.xlsx
+++ b/Test_Data/FactTable.xlsx
@@ -8,21 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/55cd0139eebd0c53/Desktop/Github Repo/PaupackLaxStatTracking/Test_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="341" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71565E1A-B9F7-4D40-82F5-248252D4BA31}"/>
+  <xr:revisionPtr revIDLastSave="342" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{99650D74-B084-410F-ACA1-B56DBBEA8042}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-5010" windowWidth="29040" windowHeight="15720" xr2:uid="{FADB34D3-2AD0-4900-91AC-1DDA22919594}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
-    <sheet name="FactTable" sheetId="2" r:id="rId2"/>
+    <sheet name="FactTable" sheetId="2" r:id="rId1"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId2"/>
   </externalReferences>
   <calcPr calcId="191029"/>
-  <pivotCaches>
-    <pivotCache cacheId="6" r:id="rId4"/>
-  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="46">
   <si>
     <t>Maplewood HS</t>
   </si>
@@ -182,48 +178,6 @@
   <si>
     <t>Lauren Scott</t>
   </si>
-  <si>
-    <t>Row Labels</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>Sum of Goals</t>
-  </si>
-  <si>
-    <t>Sum of Assists</t>
-  </si>
-  <si>
-    <t>Sum of GBs</t>
-  </si>
-  <si>
-    <t>Sum of CTOs</t>
-  </si>
-  <si>
-    <t>Sum of TOs</t>
-  </si>
-  <si>
-    <t>Sum of WomanUpGoals</t>
-  </si>
-  <si>
-    <t>Sum of WomanDownGoals</t>
-  </si>
-  <si>
-    <t>Sum of Shots</t>
-  </si>
-  <si>
-    <t>Sum of ShotsFaced</t>
-  </si>
-  <si>
-    <t>Sum of Saves</t>
-  </si>
-  <si>
-    <t>Sum of DrawAtts</t>
-  </si>
-  <si>
-    <t>Sum of DrawControls</t>
-  </si>
 </sst>
 </file>
 
@@ -295,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -306,11 +260,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -423,1684 +372,6 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Chris Napoli" refreshedDate="46084.654355555555" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="70" xr:uid="{45BECAE6-F96A-464F-B8E1-6CE7A28CF657}">
-  <cacheSource type="worksheet">
-    <worksheetSource ref="A1:R71" sheet="FactTable"/>
-  </cacheSource>
-  <cacheFields count="18">
-    <cacheField name="PlayerID" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1" maxValue="10"/>
-    </cacheField>
-    <cacheField name="F_PlayerName" numFmtId="0">
-      <sharedItems count="10">
-        <s v="Olivia Hart"/>
-        <s v="Mia Russo"/>
-        <s v="Emma Torres"/>
-        <s v="Sophie Kim"/>
-        <s v="Ava Nguyen"/>
-        <s v="Chloe Banks"/>
-        <s v="Riley Patel"/>
-        <s v="Jenna Walsh"/>
-        <s v="Natalie Cruz"/>
-        <s v="Lauren Scott"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="Date" numFmtId="0">
-      <sharedItems count="7">
-        <s v="2025-03-08"/>
-        <s v="2025-03-15"/>
-        <s v="2025-03-22"/>
-        <s v="2025-03-29"/>
-        <s v="2025-04-05"/>
-        <s v="2025-04-12"/>
-        <s v="2025-04-19"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="OpponentName" numFmtId="0">
-      <sharedItems/>
-    </cacheField>
-    <cacheField name="Goals" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
-    </cacheField>
-    <cacheField name="Assists" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="2"/>
-    </cacheField>
-    <cacheField name="Shots" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="7"/>
-    </cacheField>
-    <cacheField name="GBs" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="5"/>
-    </cacheField>
-    <cacheField name="TOs" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
-    </cacheField>
-    <cacheField name="DrawAtts" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="4"/>
-    </cacheField>
-    <cacheField name="DrawControls" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
-    </cacheField>
-    <cacheField name="ShotsFaced" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="11"/>
-    </cacheField>
-    <cacheField name="Saves" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="8" count="6">
-        <n v="0"/>
-        <n v="4"/>
-        <n v="3"/>
-        <n v="8"/>
-        <n v="1"/>
-        <n v="5"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="WomanUpGoals" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
-    </cacheField>
-    <cacheField name="WomanDownGoals" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
-    </cacheField>
-    <cacheField name="CTOs" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="3"/>
-    </cacheField>
-    <cacheField name="PenType" numFmtId="0">
-      <sharedItems containsBlank="1" count="5">
-        <m/>
-        <s v="Green"/>
-        <s v="Yellow"/>
-        <s v="12m"/>
-        <s v="Red"/>
-      </sharedItems>
-    </cacheField>
-    <cacheField name="MinsServed" numFmtId="0">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="0" maxValue="1"/>
-    </cacheField>
-  </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
-</pivotCacheDefinition>
-</file>
-
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="70">
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <x v="1"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="0"/>
-    <s v="Riverside HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="5"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="1"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="5"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="1"/>
-    <s v="Lakewood HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="8"/>
-    <x v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="2"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="3"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="2"/>
-    <s v="Northview HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="9"/>
-    <x v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="1"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="7"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="3"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="2"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="5"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="3"/>
-    <s v="Summit Academy"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="8"/>
-    <x v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="5"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="1"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="4"/>
-    <s v="Eastbrook HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="11"/>
-    <x v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="5"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="3"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="3"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="5"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <x v="2"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="5"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="5"/>
-    <s v="Cedar Falls HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="5"/>
-    <x v="4"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="3"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="1"/>
-    <x v="0"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="6"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="2"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <n v="2"/>
-    <x v="1"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="1"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="3"/>
-    <x v="2"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="4"/>
-    <x v="3"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="2"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="4"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="5"/>
-    <x v="4"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="4"/>
-    <n v="4"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="2"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="6"/>
-    <x v="5"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="1"/>
-    <n v="3"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="7"/>
-    <x v="6"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="4"/>
-    <n v="3"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="8"/>
-    <x v="7"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="9"/>
-    <x v="8"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="2"/>
-    <n v="2"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="3"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <n v="10"/>
-    <x v="9"/>
-    <x v="6"/>
-    <s v="Maplewood HS"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="1"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="10"/>
-    <x v="5"/>
-    <n v="0"/>
-    <n v="0"/>
-    <n v="0"/>
-    <x v="0"/>
-    <n v="0"/>
-  </r>
-</pivotCacheRecords>
-</file>
-
-<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{93B1F2E5-6101-4B7D-8463-217B5EDC7EF7}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A3:M14" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="18">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="11">
-        <item x="4"/>
-        <item x="5"/>
-        <item x="2"/>
-        <item x="7"/>
-        <item x="9"/>
-        <item x="1"/>
-        <item x="8"/>
-        <item x="0"/>
-        <item x="6"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="8">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0">
-      <items count="7">
-        <item x="0"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="3"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="11">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="5"/>
-    </i>
-    <i>
-      <x v="6"/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="8"/>
-    </i>
-    <i>
-      <x v="9"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
-    <field x="-2"/>
-  </colFields>
-  <colItems count="12">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-    <i i="3">
-      <x v="3"/>
-    </i>
-    <i i="4">
-      <x v="4"/>
-    </i>
-    <i i="5">
-      <x v="5"/>
-    </i>
-    <i i="6">
-      <x v="6"/>
-    </i>
-    <i i="7">
-      <x v="7"/>
-    </i>
-    <i i="8">
-      <x v="8"/>
-    </i>
-    <i i="9">
-      <x v="9"/>
-    </i>
-    <i i="10">
-      <x v="10"/>
-    </i>
-    <i i="11">
-      <x v="11"/>
-    </i>
-  </colItems>
-  <dataFields count="12">
-    <dataField name="Sum of Goals" fld="4" baseField="0" baseItem="0"/>
-    <dataField name="Sum of Assists" fld="5" baseField="0" baseItem="0"/>
-    <dataField name="Sum of GBs" fld="7" baseField="0" baseItem="0"/>
-    <dataField name="Sum of TOs" fld="8" baseField="0" baseItem="0"/>
-    <dataField name="Sum of CTOs" fld="15" baseField="0" baseItem="0"/>
-    <dataField name="Sum of Shots" fld="6" baseField="0" baseItem="0"/>
-    <dataField name="Sum of WomanUpGoals" fld="13" baseField="0" baseItem="0"/>
-    <dataField name="Sum of WomanDownGoals" fld="14" baseField="0" baseItem="0"/>
-    <dataField name="Sum of DrawAtts" fld="9" baseField="0" baseItem="0"/>
-    <dataField name="Sum of DrawControls" fld="10" baseField="0" baseItem="0"/>
-    <dataField name="Sum of ShotsFaced" fld="11" baseField="0" baseItem="0"/>
-    <dataField name="Sum of Saves" fld="12" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2419,523 +690,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EBA3C68-2291-42D7-93ED-B36167695E1B}">
-  <dimension ref="A3:M14"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.7265625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.08984375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="12.54296875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H3" t="s">
-        <v>53</v>
-      </c>
-      <c r="I3" t="s">
-        <v>54</v>
-      </c>
-      <c r="J3" t="s">
-        <v>58</v>
-      </c>
-      <c r="K3" t="s">
-        <v>59</v>
-      </c>
-      <c r="L3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B4" s="6">
-        <v>6</v>
-      </c>
-      <c r="C4" s="6">
-        <v>4</v>
-      </c>
-      <c r="D4" s="6">
-        <v>20</v>
-      </c>
-      <c r="E4" s="6">
-        <v>6</v>
-      </c>
-      <c r="F4" s="6">
-        <v>9</v>
-      </c>
-      <c r="G4" s="6">
-        <v>17</v>
-      </c>
-      <c r="H4" s="6">
-        <v>1</v>
-      </c>
-      <c r="I4" s="6">
-        <v>0</v>
-      </c>
-      <c r="J4" s="6">
-        <v>17</v>
-      </c>
-      <c r="K4" s="6">
-        <v>11</v>
-      </c>
-      <c r="L4" s="6">
-        <v>0</v>
-      </c>
-      <c r="M4" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B5" s="6">
-        <v>5</v>
-      </c>
-      <c r="C5" s="6">
-        <v>3</v>
-      </c>
-      <c r="D5" s="6">
-        <v>21</v>
-      </c>
-      <c r="E5" s="6">
-        <v>9</v>
-      </c>
-      <c r="F5" s="6">
-        <v>11</v>
-      </c>
-      <c r="G5" s="6">
-        <v>11</v>
-      </c>
-      <c r="H5" s="6">
-        <v>0</v>
-      </c>
-      <c r="I5" s="6">
-        <v>3</v>
-      </c>
-      <c r="J5" s="6">
-        <v>0</v>
-      </c>
-      <c r="K5" s="6">
-        <v>0</v>
-      </c>
-      <c r="L5" s="6">
-        <v>0</v>
-      </c>
-      <c r="M5" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A6" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="6">
-        <v>8</v>
-      </c>
-      <c r="C6" s="6">
-        <v>8</v>
-      </c>
-      <c r="D6" s="6">
-        <v>18</v>
-      </c>
-      <c r="E6" s="6">
-        <v>5</v>
-      </c>
-      <c r="F6" s="6">
-        <v>4</v>
-      </c>
-      <c r="G6" s="6">
-        <v>16</v>
-      </c>
-      <c r="H6" s="6">
-        <v>0</v>
-      </c>
-      <c r="I6" s="6">
-        <v>0</v>
-      </c>
-      <c r="J6" s="6">
-        <v>17</v>
-      </c>
-      <c r="K6" s="6">
-        <v>8</v>
-      </c>
-      <c r="L6" s="6">
-        <v>0</v>
-      </c>
-      <c r="M6" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A7" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B7" s="6">
-        <v>6</v>
-      </c>
-      <c r="C7" s="6">
-        <v>3</v>
-      </c>
-      <c r="D7" s="6">
-        <v>24</v>
-      </c>
-      <c r="E7" s="6">
-        <v>8</v>
-      </c>
-      <c r="F7" s="6">
-        <v>11</v>
-      </c>
-      <c r="G7" s="6">
-        <v>13</v>
-      </c>
-      <c r="H7" s="6">
-        <v>0</v>
-      </c>
-      <c r="I7" s="6">
-        <v>3</v>
-      </c>
-      <c r="J7" s="6">
-        <v>0</v>
-      </c>
-      <c r="K7" s="6">
-        <v>0</v>
-      </c>
-      <c r="L7" s="6">
-        <v>0</v>
-      </c>
-      <c r="M7" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A8" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="6">
-        <v>0</v>
-      </c>
-      <c r="C8" s="6">
-        <v>0</v>
-      </c>
-      <c r="D8" s="6">
-        <v>6</v>
-      </c>
-      <c r="E8" s="6">
-        <v>6</v>
-      </c>
-      <c r="F8" s="6">
-        <v>0</v>
-      </c>
-      <c r="G8" s="6">
-        <v>0</v>
-      </c>
-      <c r="H8" s="6">
-        <v>0</v>
-      </c>
-      <c r="I8" s="6">
-        <v>0</v>
-      </c>
-      <c r="J8" s="6">
-        <v>0</v>
-      </c>
-      <c r="K8" s="6">
-        <v>0</v>
-      </c>
-      <c r="L8" s="6">
-        <v>56</v>
-      </c>
-      <c r="M8" s="6">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="6">
-        <v>7</v>
-      </c>
-      <c r="C9" s="6">
-        <v>8</v>
-      </c>
-      <c r="D9" s="6">
-        <v>10</v>
-      </c>
-      <c r="E9" s="6">
-        <v>9</v>
-      </c>
-      <c r="F9" s="6">
-        <v>4</v>
-      </c>
-      <c r="G9" s="6">
-        <v>21</v>
-      </c>
-      <c r="H9" s="6">
-        <v>2</v>
-      </c>
-      <c r="I9" s="6">
-        <v>0</v>
-      </c>
-      <c r="J9" s="6">
-        <v>0</v>
-      </c>
-      <c r="K9" s="6">
-        <v>0</v>
-      </c>
-      <c r="L9" s="6">
-        <v>0</v>
-      </c>
-      <c r="M9" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B10" s="6">
-        <v>2</v>
-      </c>
-      <c r="C10" s="6">
-        <v>2</v>
-      </c>
-      <c r="D10" s="6">
-        <v>21</v>
-      </c>
-      <c r="E10" s="6">
-        <v>10</v>
-      </c>
-      <c r="F10" s="6">
-        <v>11</v>
-      </c>
-      <c r="G10" s="6">
-        <v>9</v>
-      </c>
-      <c r="H10" s="6">
-        <v>0</v>
-      </c>
-      <c r="I10" s="6">
-        <v>4</v>
-      </c>
-      <c r="J10" s="6">
-        <v>0</v>
-      </c>
-      <c r="K10" s="6">
-        <v>0</v>
-      </c>
-      <c r="L10" s="6">
-        <v>0</v>
-      </c>
-      <c r="M10" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="6">
-        <v>14</v>
-      </c>
-      <c r="C11" s="6">
-        <v>5</v>
-      </c>
-      <c r="D11" s="6">
-        <v>17</v>
-      </c>
-      <c r="E11" s="6">
-        <v>4</v>
-      </c>
-      <c r="F11" s="6">
-        <v>3</v>
-      </c>
-      <c r="G11" s="6">
-        <v>26</v>
-      </c>
-      <c r="H11" s="6">
-        <v>2</v>
-      </c>
-      <c r="I11" s="6">
-        <v>0</v>
-      </c>
-      <c r="J11" s="6">
-        <v>0</v>
-      </c>
-      <c r="K11" s="6">
-        <v>0</v>
-      </c>
-      <c r="L11" s="6">
-        <v>0</v>
-      </c>
-      <c r="M11" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="6">
-        <v>3</v>
-      </c>
-      <c r="C12" s="6">
-        <v>2</v>
-      </c>
-      <c r="D12" s="6">
-        <v>16</v>
-      </c>
-      <c r="E12" s="6">
-        <v>10</v>
-      </c>
-      <c r="F12" s="6">
-        <v>13</v>
-      </c>
-      <c r="G12" s="6">
-        <v>7</v>
-      </c>
-      <c r="H12" s="6">
-        <v>0</v>
-      </c>
-      <c r="I12" s="6">
-        <v>2</v>
-      </c>
-      <c r="J12" s="6">
-        <v>0</v>
-      </c>
-      <c r="K12" s="6">
-        <v>0</v>
-      </c>
-      <c r="L12" s="6">
-        <v>0</v>
-      </c>
-      <c r="M12" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A13" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B13" s="6">
-        <v>6</v>
-      </c>
-      <c r="C13" s="6">
-        <v>9</v>
-      </c>
-      <c r="D13" s="6">
-        <v>17</v>
-      </c>
-      <c r="E13" s="6">
-        <v>12</v>
-      </c>
-      <c r="F13" s="6">
-        <v>6</v>
-      </c>
-      <c r="G13" s="6">
-        <v>14</v>
-      </c>
-      <c r="H13" s="6">
-        <v>0</v>
-      </c>
-      <c r="I13" s="6">
-        <v>0</v>
-      </c>
-      <c r="J13" s="6">
-        <v>13</v>
-      </c>
-      <c r="K13" s="6">
-        <v>6</v>
-      </c>
-      <c r="L13" s="6">
-        <v>0</v>
-      </c>
-      <c r="M13" s="6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B14" s="6">
-        <v>57</v>
-      </c>
-      <c r="C14" s="6">
-        <v>44</v>
-      </c>
-      <c r="D14" s="6">
-        <v>170</v>
-      </c>
-      <c r="E14" s="6">
-        <v>79</v>
-      </c>
-      <c r="F14" s="6">
-        <v>72</v>
-      </c>
-      <c r="G14" s="6">
-        <v>134</v>
-      </c>
-      <c r="H14" s="6">
-        <v>5</v>
-      </c>
-      <c r="I14" s="6">
-        <v>12</v>
-      </c>
-      <c r="J14" s="6">
-        <v>47</v>
-      </c>
-      <c r="K14" s="6">
-        <v>25</v>
-      </c>
-      <c r="L14" s="6">
-        <v>56</v>
-      </c>
-      <c r="M14" s="6">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{675130FE-5529-48C3-883E-D019D34D4137}">
   <dimension ref="A1:R71"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Complete comments to code
</commit_message>
<xml_diff>
--- a/Test_Data/FactTable.xlsx
+++ b/Test_Data/FactTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/55cd0139eebd0c53/Desktop/Github Repo/PaupackLaxStatTracking/Test_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="343" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{511952F7-274B-4F44-A6D1-4DD9ACB4E69A}"/>
+  <xr:revisionPtr revIDLastSave="351" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{295C1F71-4C65-431C-8576-6E62310EB1F0}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5010" windowWidth="29040" windowHeight="15720" xr2:uid="{FADB34D3-2AD0-4900-91AC-1DDA22919594}"/>
+    <workbookView xWindow="28680" yWindow="-7935" windowWidth="29040" windowHeight="15720" xr2:uid="{FADB34D3-2AD0-4900-91AC-1DDA22919594}"/>
   </bookViews>
   <sheets>
     <sheet name="FactTable" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
Change input to google sheets url
</commit_message>
<xml_diff>
--- a/Test_Data/FactTable.xlsx
+++ b/Test_Data/FactTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/55cd0139eebd0c53/Desktop/Github Repo/PaupackLaxStatTracking/Test_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="351" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{295C1F71-4C65-431C-8576-6E62310EB1F0}"/>
+  <xr:revisionPtr revIDLastSave="352" documentId="8_{6D691F99-DFB6-41F9-ABE0-713B804467D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAEE05FA-3900-47AA-9477-21A36F027E6B}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-7935" windowWidth="29040" windowHeight="15720" xr2:uid="{FADB34D3-2AD0-4900-91AC-1DDA22919594}"/>
+    <workbookView xWindow="28680" yWindow="-5010" windowWidth="29040" windowHeight="15720" xr2:uid="{FADB34D3-2AD0-4900-91AC-1DDA22919594}"/>
   </bookViews>
   <sheets>
     <sheet name="FactTable" sheetId="2" r:id="rId1"/>
@@ -4644,5 +4644,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>